<commit_message>
Made changes to the file classifier and Summerizer.py
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,21 +460,21 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>The paper addresses the inefficiencies inherent in recurrent and convolutional sequence‑to‑sequence
-models, whose sequential computation hinders parallelism and inflates training time, especially for
-long sequences. To overcome this, the authors introduce the Transformer, an architecture that
-discards recurrence and convolution entirely, relying instead on stacked layers of multi‑head
-self‑attention and position‑wise feed‑forward networks. Central to the design are scaled dot‑product
-attention, multi‑head attention that captures information from multiple representation subspaces,
-and a parameter‑free sinusoidal positional encoding that injects order information. Experiments on
-WMT 2014 English‑German and English‑French translation tasks demonstrate that the Transformer
-achieves state‑of‑the‑art BLEU scores (28.4 and 41.8 respectively) while training up to 12 times
-faster than comparable recurrent models, requiring only a few days on eight GPUs. The model also
-generalizes to English constituency parsing, performing well with both large and limited datasets.
-The authors release their code via tensor2tensor, facilitating reproducibility and further research.
-Overall, the work establishes that attention‑only models can surpass traditional architectures in
-both quality and efficiency, opening new avenues for parallelizable sequence modeling across diverse
-domains.</t>
+          <t>The paper addresses the limitations of dominant sequence‑to‑sequence models that rely on recurrent
+or convolutional networks, which process tokens sequentially and thus hinder parallel computation
+and increase training time. To overcome this, the authors propose the Transformer architecture,
+which eliminates recurrence and convolutions entirely and builds both encoder and decoder solely
+from stacked multi‑head self‑attention layers and position‑wise feed‑forward networks, supplemented
+by learned positional encodings. By computing attention across all positions simultaneously, the
+model enables far greater parallelism, reduces the number of sequential operations, and consequently
+shortens training time while maintaining or improving translation quality. Experiments on the WMT
+2014 English‑German and English‑French benchmarks demonstrate that the Transformer achieves new
+state‑of‑the‑art BLEU scores (28.4 and 41.8 respectively) with significantly less training
+cost—training on eight GPUs for only a few days compared to weeks for prior models. The paper also
+shows that the architecture generalizes to other tasks, such as English constituency parsing, both
+with abundant and limited data. Key contributions include the introduction of scaled dot‑product
+attention, multi‑head attention, and a parameter‑free positional encoding scheme, all of which
+together enable efficient, high‑performance sequence transduction without recurrence.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -484,16 +484,16 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>The primary contribution is the design of an attention‑only architecture that eliminates sequential
-recurrence, dramatically increasing parallelism and reducing training time without increasing model
-size. The paper focuses on novel attention mechanisms (scaled dot‑product, multi‑head) and
-positional encodings rather than scaling up parameters or data. No scaling laws or massive model
-regimes are explored, placing the work squarely in the efficiency domain.</t>
+          <t>The primary contribution is an architectural redesign that replaces recurrent computation with fully
+parallelizable attention mechanisms, drastically reducing training time and computational
+bottlenecks. The paper focuses on achieving faster training and inference while preserving or
+improving accuracy, rather than scaling model size or data volume. Techniques such as multi‑head
+self‑attention and positional encodings target efficiency gains, fitting the Efficiency category.</t>
         </is>
       </c>
     </row>
@@ -505,21 +505,21 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>The paper investigates how the performance of neural language models, measured by cross‑entropy
-loss, varies systematically with three fundamental resources: model size (parameter count), dataset
-size, and the total compute expended during training. By training a broad suite of Transformer and
-LSTM models across seven orders of magnitude in each dimension, the authors discover that loss
-follows a simple power‑law relationship with each resource, with only minor deviations. They further
-derive analytic expressions that capture the onset of over‑fitting as a function of model‑to‑data
-ratio and that describe how training speed scales with model size. Using these formulas, they
-formulate an optimal allocation strategy for a fixed compute budget, showing that the most
-compute‑efficient regime involves training very large models on relatively modest data and halting
-training well before full convergence. The results demonstrate that larger models are dramatically
-more sample‑efficient, implying that traditional practices of training until convergence on massive
-datasets are suboptimal. The study also finds that architectural tweaks such as varying depth or
-width have limited impact compared to the primary scaling variables. Overall, the work provides a
-quantitative framework for predicting model performance, guiding resource planning, and highlighting
-the benefits of scaling up model size in the context of limited data and compute.</t>
+          <t>The paper investigates empirical scaling laws governing the performance of neural language models
+measured by cross‑entropy loss. It demonstrates that loss follows a power‑law relationship with
+respect to model size, dataset size, and the total compute used for training, with trends observable
+across more than seven orders of magnitude. By systematically varying these factors, the authors
+find that architectural choices such as network width or depth have relatively minor impact within
+broad ranges, allowing simple equations to capture how over‑fitting depends on model and data scale
+and how training speed varies with model size. These equations enable the optimal allocation of a
+fixed compute budget: larger models are markedly more sample‑efficient, so the most
+compute‑efficient training strategy is to train very large models on comparatively modest data and
+halt training well before full convergence. The work includes extensive experiments on both
+Transformer and LSTM architectures, leveraging an optimized Transformer implementation and curated
+text datasets. Contributions include deriving closed‑form scaling relationships, revealing that
+optimal performance arises from a compute‑driven balance rather than maximal data usage, and
+providing practical guidance for designing and training future large‑scale language models under
+resource constraints.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -529,17 +529,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>98%</t>
+          <t>96%</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>The authors empirically derive power‑law scaling relationships linking loss to model size, data
-quantity, and compute, and use these to propose optimal compute allocation strategies. Their
-methodology centers on systematic large‑scale experiments rather than introducing new efficient
-architectures or compression techniques. The primary contribution is a quantitative understanding of
-how performance scales with resources, fitting the definition of a scaling study. Consequently, the
-paper aligns with the Scaling category rather than Efficiency.</t>
+          <t>The paper’s primary focus is on quantifying how model performance scales with size, data, and
+compute, deriving power‑law relationships that predict optimal training regimes. It does not propose
+new efficiency techniques such as quantization or pruning, but rather provides a theoretical and
+empirical framework for understanding the benefits of increasing scale. The methodology relies on
+large‑scale experiments across many orders of magnitude, fitting simple equations to observed
+trends. Consequently, its contribution lies squarely in the scaling domain rather than efficiency.</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>The paper addresses the practical problem of allocating a fixed training compute budget when
-developing large language models (LLMs). While prior work (Kaplan et al., 2020) suggested that
-compute‑optimal performance is achieved by increasing model size faster than the number of training
-tokens, the authors re‑examine this trade‑off using a large empirical dataset of over 400 model runs
-spanning 70 M to 16 B parameters and 5 B to 400 B tokens. They model the final pre‑training loss
-L(N,D) as a function of parameters N and token count D, and solve for the optimal (N_opt, D_opt)
-that minimizes loss under a FLOPs constraint C. Their analysis reveals that, contrary to earlier
-scaling laws, model size and token count should be scaled proportionally: a ten‑fold increase in
-compute should be split evenly between larger models and longer training. Applying this insight,
-they train a 70 B‑parameter model named Chinchilla on 1.4 trillion tokens—four times more data and
-four times smaller than the 280 B‑parameter Gopher trained on 300 B tokens. Chinchilla outperforms
-Gopher and other contemporary LLMs despite its smaller size, offering lower inference cost and
-reduced energy consumption. The work therefore provides a revised compute‑optimal frontier for LLMs,
-challenges existing scaling prescriptions, and demonstrates the practical benefits of training
-smaller models longer.</t>
+          <t>The paper addresses how to allocate a fixed training compute budget between model size (number of
+parameters) and the amount of data (training tokens) for large language models. Building on prior
+scaling‑law work, the authors empirically model the final pre‑training loss as a function of
+parameters N and tokens D using over 400 trained models ranging from 70 M to 16 B parameters and 5 B
+to 400 B tokens. By treating FLOPs(N, D) as a deterministic budget constraint, they solve for the
+optimal (N_opt, D_opt) that minimizes loss for any given compute budget C. Their analysis diverges
+from Kaplan et al. (2020), which suggested that larger models should be trained on only modestly
+more data; instead they find that model size and token count should scale proportionally. To
+validate the revised frontier they train a 70 B‑parameter model, Chinchilla, on 1.4 trillion
+tokens—four times more data and four times fewer parameters than the 280 B‑parameter Gopher model
+trained on the same compute. Chinchilla achieves lower loss and better downstream performance while
+reducing inference cost. The key contributions are (1) a new empirically derived compute‑optimal
+scaling law, (2) a comprehensive dataset of loss measurements across many model‑size and data‑scale
+configurations, (3) the demonstration that current state‑of‑the‑art LLMs are under‑trained on data,
+and (4) the release of the Chinchilla model as a practical example of the optimal trade‑off.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -580,12 +580,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>The paper develops and validates new scaling laws for LLMs by empirically fitting loss surfaces
-across many model sizes and token budgets, then derives optimal parameter‑token trade‑offs under a
-fixed FLOPs constraint. Its primary contribution is a revised theoretical and empirical framework
-for how compute should be allocated between model capacity and data, not a novel efficiency
-technique. The introduction of the Chinchilla model serves to empirically confirm these scaling
-insights, reinforcing its classification as a scaling study.</t>
+          <t>The work focuses on deriving and validating a new scaling law that relates model size, data
+quantity, and compute, rather than introducing a novel efficiency technique. It empirically fits
+loss across many models to determine the optimal trade‑off, directly addressing how capabilities
+grow with scale. The primary novelty lies in revising the established scaling relationship (Kaplan
+et al.) and demonstrating its impact with the Chinchilla model. Thus, the main contribution is
+understanding and applying scaling behavior.</t>
         </is>
       </c>
     </row>
@@ -597,22 +597,21 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>The paper investigates the phenomenon of emergent abilities in large language models—capabilities
-that are absent in smaller models but appear abruptly once a certain scale is reached. While scaling
-laws have reliably predicted continuous performance improvements for many tasks, the authors argue
-that some abilities cannot be extrapolated from smaller models and instead manifest as qualitative
-phase‑transitions. They formalize emergence as a function of model scale measured by training
-compute (FLOPs) and parameter count, illustrating typical scaling curves where performance stays
-near random until a critical threshold, after which it rises sharply. The methodology involves
-reviewing prior empirical findings, plotting performance against compute and parameters, and
-categorizing emergent abilities observed in few‑shot prompting and augmented prompting contexts. By
-contrasting emergent behaviors with predictable scaling trends, the paper highlights that scaling
-can yield unexpected capabilities, raising questions about the limits of model growth and the
-underlying mechanisms that drive such qualitative changes. Key contributions include a precise
-definition of emergent abilities, empirical evidence of phase‑transition‑like behavior across model
-families, a taxonomy of observed emergent tasks, and a discussion of future research directions to
-understand why these abilities arise and whether further scaling will continue to produce new
-capabilities.</t>
+          <t>The paper investigates “emergent abilities” in large language models—capabilities that appear
+abruptly once model scale crosses a certain threshold and are absent in smaller models. While
+scaling laws have successfully predicted smooth performance improvements for many tasks, the authors
+argue that some abilities cannot be extrapolated from smaller models, constituting a qualitative
+change akin to a phase transition. They define emergence formally as a performance jump from
+near‑random to substantially above random at a critical scale, measured in training FLOPs or
+parameter count, and discuss how this phenomenon manifests across various tasks such as few‑shot
+prompting and augmented prompting strategies. The methodology consists of surveying prior work,
+plotting scaling curves for different models, and analyzing the relationship between compute,
+parameters, and dataset size to illustrate where emergent behaviors arise. Key contributions include
+a clear operational definition of emergent abilities, empirical visualizations that reveal abrupt
+performance shifts, and a taxonomy of observed emergent tasks. The paper also highlights open
+research questions about the underlying mechanisms driving emergence and whether continued scaling
+will yield further qualitative capabilities, thereby framing emergence as a central motivation for
+future scaling studies.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -627,11 +626,11 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>The work centers on analyzing how model performance changes with increasing compute and parameters,
-using scaling curves to identify abrupt qualitative shifts. It defines and surveys emergent
-abilities rather than proposing new efficiency techniques. The methodology relies on empirical
-scaling analysis across model families, fitting the primary focus of scaling research. Consequently,
-it aligns with the Scaling category rather than Efficiency.</t>
+          <t>The work centers on how increasing model compute and parameters leads to qualitative, unpredicted
+capabilities, analyzing scaling curves and phase‑transition‑like behavior. It does not propose new
+efficiency techniques such as pruning or quantization, but rather studies the effects of scale on
+performance. The primary methodology is empirical analysis of large‑scale models rather than
+resource reduction, placing it squarely in the scaling domain.</t>
         </is>
       </c>
     </row>
@@ -643,20 +642,20 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The paper tackles the challenge of deploying massive generative pretrained transformer (GPT) models,
-whose billions of parameters make inference costly in memory and compute. Existing compression
-efforts for such models focus largely on quantization, while pruning methods either require
-extensive retraining or become prohibitively expensive at the scale of 100 billion‑plus weights. To
-address this gap, the authors introduce SparseGPT, a one‑shot pruning technique that reformulates
-pruning as a series of very large sparse regression problems and solves them with a novel
-approximate regression solver. This approach enables uniform layer‑wise sparsity up to 60 % (both
-unstructured and semi‑structured patterns such as 2:4 and 4:8) on the largest publicly available
-GPT‑family models (OPT‑175B and BLOOM‑176B) within roughly 4.5 hours on a single GPU, without any
-fine‑tuning. Empirical results show negligible increases in perplexity and minimal loss in zero‑shot
-accuracy, and they reveal that larger models tolerate higher sparsity levels better than smaller
-ones. SparseGPT also integrates seamlessly with weight quantization pipelines. The contribution lies
-in demonstrating that accurate, large‑scale pruning can be performed efficiently in a single pass,
-opening a practical path to reduce inference cost for state‑of‑the‑art language models.</t>
+          <t>The paper addresses the challenge of deploying massive generative pretrained transformer (GPT)
+models, which can contain 175 billion parameters and demand hundreds of gigabytes of memory and many
+high‑end GPUs for inference. Existing compression work on such models has focused almost exclusively
+on quantization, while pruning—removing weights or structures—has been limited to smaller networks
+and typically requires costly retraining. The authors propose SparseGPT, the first accurate one‑shot
+pruning technique that operates efficiently on models with tens to hundreds of billions of
+parameters. SparseGPT reformulates pruning as a series of extremely large sparse regression problems
+and solves them with a novel approximate solver that can run on a single GPU in a few hours, even
+for the 175‑billion‑parameter OPT and BLOOM models. Experiments show that SparseGPT can impose
+uniform unstructured sparsity up to 60 % with negligible increase in perplexity and minimal loss in
+zero‑shot accuracy, outperforming magnitude‑based baselines that fail beyond 10‑30 % sparsity. The
+method also extends to hardware‑friendly semi‑structured patterns (2:4 and 4:8) and is compatible
+with weight quantization. The results suggest that larger models are more amenable to pruning,
+achieving substantial reductions in inference cost while preserving performance.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -671,12 +670,156 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>SparseGPT introduces a new algorithmic method—an approximate sparse regression solver—to prune
-billions of weights in one shot, directly reducing memory and compute demands at inference time. The
-technique operates on existing GPT models without retraining, focusing on compressing rather than
-enlarging model capacity. It addresses hardware‑friendly sparsity patterns and works alongside
-quantization, emphasizing cost reduction. These characteristics align the primary contribution with
-efficiency rather than scaling the model size or data.</t>
+          <t>SparseGPT introduces a novel pruning algorithm that reduces the number of active weights in
+GPT‑scale models without any retraining, directly lowering memory usage and compute at inference
+time. The technique relies on an approximate sparse regression solver to handle billions of
+parameters efficiently on a single GPU. By achieving 50‑60 % sparsity with negligible accuracy loss,
+the work focuses on making existing large models more computationally efficient rather than scaling
+model size or data. Consequently, its primary contribution lies in efficiency improvements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>QLORA:  Efficient Finetuning of Quantized LLMs</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>The paper addresses the prohibitive memory and compute costs of fine‑tuning very large language
+models (LLMs), exemplified by a 65 billion‑parameter LLaMA model that would normally require over
+780 GB of GPU memory for 16‑bit training. QLoRA (Quantized Low‑Rank Adaptation) solves this problem
+by keeping the pretrained model frozen in a 4‑bit quantized representation while back‑propagating
+gradients only through low‑rank adapter modules (LoRA). The authors introduce three key innovations:
+(a) NF4, a 4‑bit NormalFloat data type that is information‑theoretically optimal for normally
+distributed weights, (b) Double Quantization, which compresses the quantization constants themselves
+to further reduce memory, and (c) Paged Optimizers, which dynamically allocate optimizer state to
+handle memory spikes during training. Using these techniques, QLoRA can fine‑tune a 65 B model on a
+single 48 GB GPU in about 24 hours while achieving performance comparable to full 16‑bit
+fine‑tuning. The resulting model family, named Guanaco, outperforms all publicly released models on
+the Vicuna benchmark, reaching 99.3 % of ChatGPT’s performance. Extensive experiments across eight
+instruction datasets, multiple model architectures (LLaMA, T5), and scales up to 65 B parameters
+demonstrate that high‑quality, small‑scale instruction data combined with QLoRA yields
+state‑of‑the‑art results. The paper also provides analysis of human versus GPT‑4 evaluation,
+highlighting limitations of current chatbot benchmarks, and releases code, models, and custom CUDA
+kernels for 4‑bit training.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>96%</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>The primary contribution is a set of memory‑saving techniques that enable fine‑tuning of massive
+LLMs on modest hardware, not an exploration of scaling laws or larger model sizes. QLoRA combines
+4‑bit NF4 quantization, double quantization of scale factors, and paged optimizer state to
+dramatically reduce GPU memory while preserving full‑precision performance. The work focuses on
+reducing computational footprint and training cost rather than increasing model capacity, aligning
+it with the Efficiency category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Efficient Transformers: A Survey</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Transformers have become a dominant architecture across language, vision, and retrieval tasks, yet
+their self‑attention mechanism incurs quadratic time and memory costs that limit scalability to long
+sequences and resource‑constrained environments. This survey addresses the burgeoning body of
+research that seeks to mitigate these costs, grouping the proposed models under the umbrella of
+“efficient Transformers.” The authors first define efficiency in terms of memory footprint and
+computational operations, emphasizing scenarios where inputs are large, such as documents,
+high‑resolution images, or video frames. A taxonomy is introduced that classifies models by the core
+technical innovation—such as sparse or low‑rank attention, pooling, kernel‑level optimizations, and
+parameter‑sharing schemes—and by their primary application domain. The paper then provides detailed
+walkthroughs of numerous architectures, drawing connections among them and highlighting how each
+tackles the quadratic bottleneck. In addition to attention‑centric methods, the survey briefly
+surveys orthogonal approaches like quantization, pruning, and distillation that further improve
+runtime and hardware utilization. The authors also discuss evaluation practices and emerging design
+trends, offering a consolidated view of the field that can guide future research and practical
+deployment of Transformers on long inputs or limited hardware. By synthesizing recent advances up to
+August 2020, the work serves as a timely reference for both academic and industry practitioners
+interested in reducing the computational and memory demands of Transformer models.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>The paper’s primary contribution is a comprehensive taxonomy and analysis of methods that reduce the
+quadratic complexity of self‑attention, including sparse, low‑rank, and pooling‑based techniques, as
+well as other hardware‑friendly optimizations. It focuses on lowering memory and FLOP requirements
+rather than increasing model size or data volume. The survey synthesizes efficiency‑oriented
+innovations across language and vision domains, positioning it squarely within the Efficiency
+category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FLASH ATTENTION : Fast and Memory-Efﬁcient Exact Attention with IO-Awareness</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Transformers suffer from quadratic time and memory costs in self‑attention, which hampers their use
+on long sequences. The paper identifies that existing approximate attention methods focus on FLOP
+reduction while neglecting memory‑access overheads, leading to limited wall‑clock gains. To address
+this, the authors introduce FLASHATTENTION, an IO‑aware exact attention algorithm that explicitly
+accounts for reads and writes between GPU high‑bandwidth memory (HBM) and on‑chip SRAM. By
+partitioning the Q, K, V matrices into tiles that fit in SRAM, the method minimizes costly HBM
+traffic and performs the bulk of computation on the faster on‑chip memory. The authors analytically
+derive the IO complexity, showing FLASHATTENTION requires fewer HBM accesses than standard attention
+and is optimal for a range of SRAM capacities. They further extend the approach to block‑sparse
+attention, yielding an approximate algorithm that outperforms existing sparse methods in speed.
+Empirically, FLASHATTENTION delivers up to 15 % end‑to‑end training speedup for BERT‑large
+(seq 512), a 3× acceleration for GPT‑2 (seq 1 K), and a 2.4× gain on Long‑Range Arena (seq 1 K–4 K).
+The improved efficiency enables longer context windows, resulting in better perplexity on GPT‑2 and
+higher classification accuracy on long‑document tasks, and achieves the first transformer models
+with above‑chance performance on the Path‑X and Path‑256 challenges (seq 16 K–64 K). The work
+demonstrates that IO‑aware algorithm design can provide substantial practical speedups without
+sacrificing model quality.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>The paper’s primary contribution is an algorithmic redesign of self‑attention that reduces memory
+traffic between HBM and SRAM, a classic efficiency improvement. It introduces tiling and IO‑aware
+analysis to achieve optimal HBM accesses, and extends this to a block‑sparse variant for faster
+approximate attention. The reported speedups and ability to handle longer sequences stem from these
+efficiency gains rather than scaling model size or data, placing the work firmly in the Efficiency
+category.</t>
         </is>
       </c>
     </row>

</xml_diff>